<commit_message>
Excel deck: fix four cards from the content audit, update docs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LYGqvUvY24SqANJMruMqxX
</commit_message>
<xml_diff>
--- a/content/fde-flashcards/xl/Excel Flashcards.xlsx
+++ b/content/fde-flashcards/xl/Excel Flashcards.xlsx
@@ -5191,7 +5191,7 @@
       </c>
       <c r="AN15" s="19" t="inlineStr">
         <is>
-          <t>Click row 1 and then Freeze Panes with C5 selected by mistake</t>
+          <t>Click C5 by mistake &gt; View tab &gt; Freeze Panes &gt; Freeze Panes (rows 1 to 4 and columns A and B freeze, not just the heading row)</t>
         </is>
       </c>
       <c r="AO15" s="19" t="inlineStr">
@@ -7948,7 +7948,7 @@
       </c>
       <c r="AL24" s="18" t="inlineStr">
         <is>
-          <t>IFERROR vs IFNA: IFERROR catches every error type, while IFNA catches only #N/A, so IFNA is safer when you only expect a missing lookup.</t>
+          <t>IFERROR vs IFNA: IFERROR catches every error type, while IFNA (Excel 2013 or later) catches only #N/A, so IFNA is safer when you only expect a missing lookup.</t>
         </is>
       </c>
       <c r="AM24" s="18" t="inlineStr">
@@ -7959,15 +7959,15 @@
       <c r="AN24" s="19" t="inlineStr">
         <is>
           <t>A1: 10
-B1: 0
-C1: =IFERROR("Error",A1/B1)</t>
+B1: 2
+C1: =IFERROR("Error",A1/B1) (always shows Error, even though 10/2 works)</t>
         </is>
       </c>
       <c r="AO24" s="19" t="inlineStr">
         <is>
           <t>A1: 10
-B1: 0
-C1: =IFERROR(A1/B1,"Error")</t>
+B1: 2
+C1: =IFERROR(A1/B1,"Error") (shows 5)</t>
         </is>
       </c>
       <c r="AP24" s="18" t="inlineStr">
@@ -9691,7 +9691,7 @@
 B1: 50
 B2: 70
 B3: 60
-D1: =INDEX(B1:B3,MATCH("Ravi",A1:A3))</t>
+D1: =INDEX(B1:B3,MATCH("Ravi",A1:A3)) (match_type defaults to 1, an approximate match that assumes A1:A3 is sorted A to Z; on this unsorted list it can return the wrong row)</t>
         </is>
       </c>
       <c r="AO29" s="19" t="inlineStr">
@@ -11099,7 +11099,7 @@
       <c r="BM33" s="17" t="n"/>
       <c r="BN33" s="17" t="n"/>
     </row>
-    <row r="34" ht="81" customHeight="1">
+    <row r="34" ht="108" customHeight="1">
       <c r="A34" s="17" t="inlineStr">
         <is>
           <t>XL-032</t>
@@ -11208,7 +11208,7 @@
       </c>
       <c r="V34" s="18" t="inlineStr">
         <is>
-          <t>TEXT takes a value and a format code in quotes. It returns text that looks the way the code says, so 0.00 means two decimals and 0% means percentage. The result is text, so you cannot add it up like a number.</t>
+          <t>TEXT takes a value and a format code in quotes. It returns text that looks the way the code says, so 0.00 means two decimals and 0% means percentage. The result is text, so you cannot add it up like a number. Format codes such as dd-mm-yyyy and dddd are for English-language Excel; other languages use their own codes.</t>
         </is>
       </c>
       <c r="W34" s="18" t="inlineStr">
@@ -13748,7 +13748,7 @@
       </c>
       <c r="V42" s="18" t="inlineStr">
         <is>
-          <t>Power Query opens its own editor where each action becomes a step in the Applied Steps list on the right. When you choose Close &amp; Load, the result is written to a sheet as a table. Your original data is not changed.</t>
+          <t>Power Query opens its own editor where each action becomes a step in the Applied Steps list on the right. When you choose Close &amp; Load, the result is written to a sheet as a table. Your original values are not changed, although From Table/Range first turns the range into an Excel Table.</t>
         </is>
       </c>
       <c r="W42" s="18" t="inlineStr">
@@ -13832,7 +13832,7 @@
       </c>
       <c r="AK42" s="18" t="inlineStr">
         <is>
-          <t>✗ Power Query changes my original data table → ✓ It reads the source and writes a new result table, so the original data stays as it was</t>
+          <t>✗ Power Query changes my original data → ✓ It reads the source and writes a new result table; the source values stay the same (From Table/Range only turns the range into an Excel Table first)</t>
         </is>
       </c>
       <c r="AL42" s="18" t="inlineStr">
@@ -14236,7 +14236,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="40.5" customHeight="1">
+    <row r="26" ht="54" customHeight="1">
       <c r="A26" s="24" t="inlineStr">
         <is>
           <t>Explanation</t>
@@ -14434,7 +14434,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="30" customHeight="1">
+    <row r="44" ht="108" customHeight="1">
       <c r="A44" s="24" t="inlineStr">
         <is>
           <t>Wrong code</t>
@@ -15888,7 +15888,7 @@
 AVOID / DON'T:
 Do not freeze too many rows or columns, because the frozen part can fill the whole screen on a small phone or laptop.
 WRONG CODE:
-Click row 1 and then Freeze Panes with C5 selected by mistake
+Click C5 by mistake &gt; View tab &gt; Freeze Panes &gt; Freeze Panes (rows 1 to 4 and columns A and B freeze, not just the heading row)
 RIGHT CODE:
 View tab &gt; Freeze Panes &gt; Freeze Top Row (or click A2 and choose Freeze Panes)
 MEMORY TRICK:
@@ -16662,17 +16662,17 @@
 COMMON MISTAKE:
 ✗ IFERROR fixes the real problem in the formula → ✓ IFERROR only hides the error message; the wrong data or formula is still there
 COMMONLY CONFUSED WITH:
-IFERROR vs IFNA: IFERROR catches every error type, while IFNA catches only #N/A, so IFNA is safer when you only expect a missing lookup.
+IFERROR vs IFNA: IFERROR catches every error type, while IFNA (Excel 2013 or later) catches only #N/A, so IFNA is safer when you only expect a missing lookup.
 AVOID / DON'T:
 Do not wrap a whole big formula in IFERROR without testing it first, because it can hide real mistakes.
 WRONG CODE:
 A1: 10
-B1: 0
-C1: =IFERROR("Error",A1/B1)
+B1: 2
+C1: =IFERROR("Error",A1/B1) (always shows Error, even though 10/2 works)
 RIGHT CODE:
 A1: 10
-B1: 0
-C1: =IFERROR(A1/B1,"Error")
+B1: 2
+C1: =IFERROR(A1/B1,"Error") (shows 5)
 MEMORY TRICK:
 Try first, rescue second: formula first, fallback second.
 REAL LIFE: PROJECT / WORK:
@@ -17282,7 +17282,7 @@
 B1: 50
 B2: 70
 B3: 60
-D1: =INDEX(B1:B3,MATCH("Ravi",A1:A3))
+D1: =INDEX(B1:B3,MATCH("Ravi",A1:A3)) (match_type defaults to 1, an approximate match that assumes A1:A3 is sorted A to Z; on this unsorted list it can return the wrong row)
 RIGHT CODE:
 A1: Asha
 A2: Ravi
@@ -17734,7 +17734,7 @@
 B2 shows 26%
 B3 shows 15-08-2024
 EXPLANATION:
-TEXT takes a value and a format code in quotes. It returns text that looks the way the code says, so 0.00 means two decimals and 0% means percentage. The result is text, so you cannot add it up like a number.
+TEXT takes a value and a format code in quotes. It returns text that looks the way the code says, so 0.00 means two decimals and 0% means percentage. The result is text, so you cannot add it up like a number. Format codes such as dd-mm-yyyy and dddd are for English-language Excel; other languages use their own codes.
 SIMPLE EXPLANATION (HINGLISH):
 TEXT ka kaam hai number ya date ko aapke pasand ke style me dikhana. Jaise 0.256 ko 26% likhna. Lekin result text ban jata hai, isliye uspar sum nahi chalta.
 REAL-LIFE ANALOGY:
@@ -18517,7 +18517,7 @@
 OUTPUT:
 A new sheet shows a table with three names: Asha, Ravi and Meena
 EXPLANATION:
-Power Query opens its own editor where each action becomes a step in the Applied Steps list on the right. When you choose Close &amp; Load, the result is written to a sheet as a table. Your original data is not changed.
+Power Query opens its own editor where each action becomes a step in the Applied Steps list on the right. When you choose Close &amp; Load, the result is written to a sheet as a table. Your original values are not changed, although From Table/Range first turns the range into an Excel Table.
 SIMPLE EXPLANATION (HINGLISH):
 Power Query me aap ek baar saaf karne ke steps banate ho, aur Excel unhe yaad rakhta hai. Agli baar naya data aaye to Refresh All dabao aur wahi saare steps dobara chal jate hain.
 REAL-LIFE ANALOGY:
@@ -18556,7 +18556,7 @@
 MINI CONVERSATION:
 A: Every month I get a new export and clean the same columns by hand. | B: Record the clean-up in Power Query once, and next month just click Refresh All.
 COMMON MISTAKE:
-✗ Power Query changes my original data table → ✓ It reads the source and writes a new result table, so the original data stays as it was
+✗ Power Query changes my original data → ✓ It reads the source and writes a new result table; the source values stay the same (From Table/Range only turns the range into an Excel Table first)
 COMMONLY CONFUSED WITH:
 Power Query vs a macro: Power Query records data-cleaning steps that refresh with new data, while a macro (VBA) records any clicks and keystrokes in Excel as code.
 AVOID / DON'T:

</xml_diff>